<commit_message>
bo sung, sua doi chuc nang hien thi
</commit_message>
<xml_diff>
--- a/game_theo_chu_de.xlsx
+++ b/game_theo_chu_de.xlsx
@@ -1,30 +1,14 @@
 
-<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
-<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <Application>SheetJS</Application>
-  <HeadingPairs>
-    <vt:vector size="2" baseType="variant">
-      <vt:variant>
-        <vt:lpstr>Worksheets</vt:lpstr>
-      </vt:variant>
-      <vt:variant>
-        <vt:i4>1</vt:i4>
-      </vt:variant>
-    </vt:vector>
-  </HeadingPairs>
-  <TitlesOfParts>
-    <vt:vector size="1" baseType="lpstr">
-      <vt:lpstr>Game theo chủ đề</vt:lpstr>
-    </vt:vector>
-  </TitlesOfParts>
-</Properties>
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <workbookPr codeName="ThisWorkbook"/>
+  <sheets>
+    <sheet name="Game theo chủ đề" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
 </file>
 
-<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
-<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance"/>
-</file>
-
-<file path=xl\metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
 <metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
@@ -46,7 +30,7 @@
 </metadata>
 </file>
 
-<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
   <numFmts count="1">
     <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
@@ -91,7 +75,7 @@
 </styleSheet>
 </file>
 
-<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -411,54 +395,34 @@
 </a:theme>
 </file>
 
-<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
-  <sheets>
-    <sheet name="Game theo chủ đề" sheetId="1" r:id="rId1"/>
-  </sheets>
-</workbook>
-</file>
-
-<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I315"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="35.83203125" customWidth="1"/>
-    <col min="6" max="6" width="40.83203125" customWidth="1"/>
-    <col min="7" max="7" width="50.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="50.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
         <v>Chủ đề</v>
       </c>
       <c r="B1" t="str">
-        <v xml:space="preserve">Những từ vựng sử dụng </v>
+        <v>Những từ vựng sử dụng</v>
       </c>
       <c r="C1" t="str">
-        <v>Tên Trò chơi (Trên Web)</v>
+        <v>Tên trò chơi</v>
       </c>
       <c r="D1" t="str">
-        <v>Công cụ Tạo Game</v>
+        <v>Công nghệ sử dụng</v>
       </c>
       <c r="E1" t="str">
-        <v>Loại GAME</v>
+        <v>Dạng trò chơi</v>
       </c>
       <c r="F1" t="str">
-        <v>Mục tiêu Sư phạm</v>
+        <v>Mục tiêu sư phạm</v>
       </c>
       <c r="G1" t="str">
-        <v>Gợi ý Ứng dụng</v>
+        <v>Cách thức sử dụng</v>
       </c>
       <c r="H1" t="str">
-        <v xml:space="preserve">Gợi ý Hoạt động </v>
+        <v>Tương tác</v>
       </c>
       <c r="I1" t="str">
         <v>LINK SẢN PHẨM (BẮT BUỘC)</v>
@@ -9572,134 +9536,134 @@
     </row>
   </sheetData>
   <mergeCells count="128">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="C2:C5"/>
-    <mergeCell ref="D2:D5"/>
-    <mergeCell ref="E2:E5"/>
-    <mergeCell ref="F2:F5"/>
-    <mergeCell ref="G2:G5"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="I2:I5"/>
-    <mergeCell ref="A6:A40"/>
-    <mergeCell ref="C6:C40"/>
-    <mergeCell ref="D6:D40"/>
-    <mergeCell ref="E6:E40"/>
-    <mergeCell ref="F6:F40"/>
-    <mergeCell ref="G6:G40"/>
-    <mergeCell ref="H6:H40"/>
-    <mergeCell ref="I6:I40"/>
-    <mergeCell ref="A41:A77"/>
-    <mergeCell ref="C41:C77"/>
-    <mergeCell ref="D41:D77"/>
-    <mergeCell ref="E41:E77"/>
-    <mergeCell ref="F41:F77"/>
-    <mergeCell ref="G41:G77"/>
-    <mergeCell ref="H41:H77"/>
-    <mergeCell ref="I41:I77"/>
-    <mergeCell ref="A78:A116"/>
-    <mergeCell ref="C78:C116"/>
-    <mergeCell ref="D78:D116"/>
-    <mergeCell ref="E78:E116"/>
-    <mergeCell ref="F78:F116"/>
-    <mergeCell ref="G78:G116"/>
-    <mergeCell ref="H78:H116"/>
-    <mergeCell ref="I78:I116"/>
-    <mergeCell ref="A117:A142"/>
-    <mergeCell ref="C117:C142"/>
-    <mergeCell ref="D117:D142"/>
-    <mergeCell ref="E117:E142"/>
-    <mergeCell ref="F117:F142"/>
-    <mergeCell ref="G117:G142"/>
-    <mergeCell ref="H117:H142"/>
-    <mergeCell ref="I117:I142"/>
-    <mergeCell ref="A143:A158"/>
-    <mergeCell ref="C143:C158"/>
-    <mergeCell ref="D143:D158"/>
-    <mergeCell ref="E143:E158"/>
-    <mergeCell ref="F143:F158"/>
-    <mergeCell ref="G143:G158"/>
-    <mergeCell ref="H143:H158"/>
-    <mergeCell ref="I143:I158"/>
-    <mergeCell ref="A159:A178"/>
-    <mergeCell ref="C159:C178"/>
-    <mergeCell ref="D159:D178"/>
-    <mergeCell ref="E159:E178"/>
-    <mergeCell ref="F159:F178"/>
-    <mergeCell ref="G159:G178"/>
-    <mergeCell ref="H159:H178"/>
-    <mergeCell ref="I159:I178"/>
-    <mergeCell ref="A179:A192"/>
-    <mergeCell ref="C179:C192"/>
-    <mergeCell ref="D179:D192"/>
-    <mergeCell ref="E179:E192"/>
-    <mergeCell ref="F179:F192"/>
-    <mergeCell ref="G179:G192"/>
-    <mergeCell ref="H179:H192"/>
-    <mergeCell ref="I179:I192"/>
-    <mergeCell ref="A193:A197"/>
-    <mergeCell ref="C193:C197"/>
-    <mergeCell ref="D193:D197"/>
-    <mergeCell ref="E193:E197"/>
-    <mergeCell ref="F193:F197"/>
-    <mergeCell ref="G193:G197"/>
-    <mergeCell ref="H193:H197"/>
-    <mergeCell ref="I193:I197"/>
-    <mergeCell ref="A198:A217"/>
-    <mergeCell ref="C198:C217"/>
-    <mergeCell ref="D198:D217"/>
-    <mergeCell ref="E198:E217"/>
-    <mergeCell ref="F198:F217"/>
-    <mergeCell ref="G198:G217"/>
-    <mergeCell ref="H198:H217"/>
-    <mergeCell ref="I198:I217"/>
-    <mergeCell ref="A218:A244"/>
-    <mergeCell ref="C218:C244"/>
-    <mergeCell ref="D218:D244"/>
-    <mergeCell ref="E218:E244"/>
-    <mergeCell ref="F218:F244"/>
-    <mergeCell ref="G218:G244"/>
-    <mergeCell ref="H218:H244"/>
-    <mergeCell ref="I218:I244"/>
-    <mergeCell ref="A245:A254"/>
-    <mergeCell ref="C245:C254"/>
-    <mergeCell ref="D245:D254"/>
-    <mergeCell ref="E245:E254"/>
-    <mergeCell ref="F245:F254"/>
-    <mergeCell ref="G245:G254"/>
-    <mergeCell ref="H245:H254"/>
-    <mergeCell ref="I245:I254"/>
-    <mergeCell ref="A255:A272"/>
-    <mergeCell ref="C255:C272"/>
-    <mergeCell ref="D255:D272"/>
-    <mergeCell ref="E255:E272"/>
-    <mergeCell ref="F255:F272"/>
-    <mergeCell ref="G255:G272"/>
-    <mergeCell ref="H255:H272"/>
-    <mergeCell ref="I255:I272"/>
-    <mergeCell ref="A273:A287"/>
-    <mergeCell ref="C273:C287"/>
-    <mergeCell ref="D273:D287"/>
-    <mergeCell ref="E273:E287"/>
-    <mergeCell ref="F273:F287"/>
-    <mergeCell ref="G273:G287"/>
-    <mergeCell ref="H273:H287"/>
-    <mergeCell ref="I273:I287"/>
-    <mergeCell ref="A288:A306"/>
-    <mergeCell ref="C288:C306"/>
-    <mergeCell ref="D288:D306"/>
-    <mergeCell ref="E288:E306"/>
-    <mergeCell ref="F288:F306"/>
-    <mergeCell ref="G288:G306"/>
-    <mergeCell ref="H288:H306"/>
-    <mergeCell ref="I288:I306"/>
-    <mergeCell ref="A307:A315"/>
-    <mergeCell ref="C307:C315"/>
-    <mergeCell ref="D307:D315"/>
-    <mergeCell ref="E307:E315"/>
-    <mergeCell ref="F307:F315"/>
-    <mergeCell ref="G307:G315"/>
-    <mergeCell ref="H307:H315"/>
-    <mergeCell ref="I307:I315"/>
+    <mergeCell ref="A2:A38"/>
+    <mergeCell ref="C2:C38"/>
+    <mergeCell ref="D2:D38"/>
+    <mergeCell ref="E2:E38"/>
+    <mergeCell ref="F2:F38"/>
+    <mergeCell ref="G2:G38"/>
+    <mergeCell ref="H2:H38"/>
+    <mergeCell ref="I2:I38"/>
+    <mergeCell ref="A39:A43"/>
+    <mergeCell ref="C39:C43"/>
+    <mergeCell ref="D39:D43"/>
+    <mergeCell ref="E39:E43"/>
+    <mergeCell ref="F39:F43"/>
+    <mergeCell ref="G39:G43"/>
+    <mergeCell ref="H39:H43"/>
+    <mergeCell ref="I39:I43"/>
+    <mergeCell ref="A44:A47"/>
+    <mergeCell ref="C44:C47"/>
+    <mergeCell ref="D44:D47"/>
+    <mergeCell ref="E44:E47"/>
+    <mergeCell ref="F44:F47"/>
+    <mergeCell ref="G44:G47"/>
+    <mergeCell ref="H44:H47"/>
+    <mergeCell ref="I44:I47"/>
+    <mergeCell ref="A48:A66"/>
+    <mergeCell ref="C48:C66"/>
+    <mergeCell ref="D48:D66"/>
+    <mergeCell ref="E48:E66"/>
+    <mergeCell ref="F48:F66"/>
+    <mergeCell ref="G48:G66"/>
+    <mergeCell ref="H48:H66"/>
+    <mergeCell ref="I48:I66"/>
+    <mergeCell ref="A67:A86"/>
+    <mergeCell ref="C67:C86"/>
+    <mergeCell ref="D67:D86"/>
+    <mergeCell ref="E67:E86"/>
+    <mergeCell ref="F67:F86"/>
+    <mergeCell ref="G67:G86"/>
+    <mergeCell ref="H67:H86"/>
+    <mergeCell ref="I67:I86"/>
+    <mergeCell ref="A87:A106"/>
+    <mergeCell ref="C87:C106"/>
+    <mergeCell ref="D87:D106"/>
+    <mergeCell ref="E87:E106"/>
+    <mergeCell ref="F87:F106"/>
+    <mergeCell ref="G87:G106"/>
+    <mergeCell ref="H87:H106"/>
+    <mergeCell ref="I87:I106"/>
+    <mergeCell ref="A107:A133"/>
+    <mergeCell ref="C107:C133"/>
+    <mergeCell ref="D107:D133"/>
+    <mergeCell ref="E107:E133"/>
+    <mergeCell ref="F107:F133"/>
+    <mergeCell ref="G107:G133"/>
+    <mergeCell ref="H107:H133"/>
+    <mergeCell ref="I107:I133"/>
+    <mergeCell ref="A134:A143"/>
+    <mergeCell ref="C134:C143"/>
+    <mergeCell ref="D134:D143"/>
+    <mergeCell ref="E134:E143"/>
+    <mergeCell ref="F134:F143"/>
+    <mergeCell ref="G134:G143"/>
+    <mergeCell ref="H134:H143"/>
+    <mergeCell ref="I134:I143"/>
+    <mergeCell ref="A144:A157"/>
+    <mergeCell ref="C144:C157"/>
+    <mergeCell ref="D144:D157"/>
+    <mergeCell ref="E144:E157"/>
+    <mergeCell ref="F144:F157"/>
+    <mergeCell ref="G144:G157"/>
+    <mergeCell ref="H144:H157"/>
+    <mergeCell ref="I144:I157"/>
+    <mergeCell ref="A158:A183"/>
+    <mergeCell ref="C158:C183"/>
+    <mergeCell ref="D158:D183"/>
+    <mergeCell ref="E158:E183"/>
+    <mergeCell ref="F158:F183"/>
+    <mergeCell ref="G158:G183"/>
+    <mergeCell ref="H158:H183"/>
+    <mergeCell ref="I158:I183"/>
+    <mergeCell ref="A184:A198"/>
+    <mergeCell ref="C184:C198"/>
+    <mergeCell ref="D184:D198"/>
+    <mergeCell ref="E184:E198"/>
+    <mergeCell ref="F184:F198"/>
+    <mergeCell ref="G184:G198"/>
+    <mergeCell ref="H184:H198"/>
+    <mergeCell ref="I184:I198"/>
+    <mergeCell ref="A199:A216"/>
+    <mergeCell ref="C199:C216"/>
+    <mergeCell ref="D199:D216"/>
+    <mergeCell ref="E199:E216"/>
+    <mergeCell ref="F199:F216"/>
+    <mergeCell ref="G199:G216"/>
+    <mergeCell ref="H199:H216"/>
+    <mergeCell ref="I199:I216"/>
+    <mergeCell ref="A217:A251"/>
+    <mergeCell ref="C217:C251"/>
+    <mergeCell ref="D217:D251"/>
+    <mergeCell ref="E217:E251"/>
+    <mergeCell ref="F217:F251"/>
+    <mergeCell ref="G217:G251"/>
+    <mergeCell ref="H217:H251"/>
+    <mergeCell ref="I217:I251"/>
+    <mergeCell ref="A252:A290"/>
+    <mergeCell ref="C252:C290"/>
+    <mergeCell ref="D252:D290"/>
+    <mergeCell ref="E252:E290"/>
+    <mergeCell ref="F252:F290"/>
+    <mergeCell ref="G252:G290"/>
+    <mergeCell ref="H252:H290"/>
+    <mergeCell ref="I252:I290"/>
+    <mergeCell ref="A291:A299"/>
+    <mergeCell ref="C291:C299"/>
+    <mergeCell ref="D291:D299"/>
+    <mergeCell ref="E291:E299"/>
+    <mergeCell ref="F291:F299"/>
+    <mergeCell ref="G291:G299"/>
+    <mergeCell ref="H291:H299"/>
+    <mergeCell ref="I291:I299"/>
+    <mergeCell ref="A300:A315"/>
+    <mergeCell ref="C300:C315"/>
+    <mergeCell ref="D300:D315"/>
+    <mergeCell ref="E300:E315"/>
+    <mergeCell ref="F300:F315"/>
+    <mergeCell ref="G300:G315"/>
+    <mergeCell ref="H300:H315"/>
+    <mergeCell ref="I300:I315"/>
   </mergeCells>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:I315"/>

</xml_diff>

<commit_message>
nang cap he thong lan 4
</commit_message>
<xml_diff>
--- a/game_theo_chu_de.xlsx
+++ b/game_theo_chu_de.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\BRAVO 15\Downloads\game tieng trung hsk 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{482C19DC-E1D5-4628-8485-143E0C9E3BC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B5A21F4-CA0B-4230-B15A-A11636339471}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="HSK 2 Topics Used" sheetId="1" r:id="rId1"/>
+    <sheet name="Game theo chủ đề" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="53">
   <si>
     <t>Chủ đề</t>
   </si>
@@ -28,28 +28,324 @@
     <t>Những từ vựng sử dụng</t>
   </si>
   <si>
-    <t>Tên trò chơi</t>
-  </si>
-  <si>
-    <t>Công nghệ sử dụng</t>
-  </si>
-  <si>
-    <t>Dạng trò chơi</t>
-  </si>
-  <si>
-    <t>Mục tiêu sư phạm</t>
-  </si>
-  <si>
-    <t>Cách thức sử dụng</t>
-  </si>
-  <si>
-    <t>Tương tác</t>
+    <t>Tên Trò chơi (Trên Web)</t>
+  </si>
+  <si>
+    <t>Công cụ Tạo Game</t>
+  </si>
+  <si>
+    <t>TV Phụ trách</t>
+  </si>
+  <si>
+    <t>Loại GAME</t>
   </si>
   <si>
     <t>LINK SẢN PHẨM (BẮT BUỘC)</t>
   </si>
   <si>
+    <t>Mục tiêu Sư phạm</t>
+  </si>
+  <si>
+    <t>Gợi ý Ứng dụng</t>
+  </si>
+  <si>
+    <t>Gợi ý Hoạt động</t>
+  </si>
+  <si>
+    <t>Con người &amp; Các mối quan hệ</t>
+  </si>
+  <si>
+    <t>Ai Là Triệu Phú HSK 2</t>
+  </si>
+  <si>
+    <t>HTML, CSS, Javascript</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Trắc nghiệm / Trò chơi truyền hình</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude1</t>
+  </si>
+  <si>
+    <t>Nhận diện Hán tự, Ghi nhớ nghĩa, Phản xạ từ vựng HSK 2</t>
+  </si>
+  <si>
+    <t>Khởi động 5 phút đầu giờ; Bài tập về nhà; Ôn tập cuối chương</t>
+  </si>
+  <si>
+    <t>Cá nhân, Chia đội thi đấu (Đội nào giành được nhiều tiền hơn), Giáo viên chiếu bảng lớp học</t>
+  </si>
+  <si>
+    <t>Cơ thể &amp; Sức khỏe</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude2</t>
+  </si>
+  <si>
+    <t>Cảm xúc &amp; Thái độ</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude3</t>
+  </si>
+  <si>
+    <t>Đời sống sinh hoạt</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude4</t>
+  </si>
+  <si>
+    <t>Đồ vật &amp; Công cụ</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude5</t>
+  </si>
+  <si>
+    <t>Địa điểm &amp; Nơi chốn</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude6</t>
+  </si>
+  <si>
+    <t>Giao thông &amp; Di chuyển</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude7</t>
+  </si>
+  <si>
+    <t>Không gian &amp; Vị trí</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude8</t>
+  </si>
+  <si>
+    <t>Thời gian</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude9</t>
+  </si>
+  <si>
+    <t>Miêu tả &amp; Đánh giá</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude10</t>
+  </si>
+  <si>
     <t>Công cụ ngữ pháp &amp; Cấu trúc</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude11</t>
+  </si>
+  <si>
+    <t>Tự nhiên</t>
+  </si>
+  <si>
+    <t>game.html?topic=chude12</t>
+  </si>
+  <si>
+    <t>介绍
+奶奶
+男孩儿
+女孩儿
+妻子
+小孩儿
+姓
+姓名
+爷爷
+丈夫</t>
+  </si>
+  <si>
+    <t>白色
+帮
+长
+高
+个子
+介绍
+累
+身体
+手
+手表
+疼
+头
+眼睛
+药
+药店</t>
+  </si>
+  <si>
+    <t>啊
+爱好
+不错
+不好意思
+坏
+快乐
+没意思
+舒服
+希望
+笑</t>
+  </si>
+  <si>
+    <t>爱情片
+帮忙
+包
+笔
+打
+打开
+蛋糕
+等
+点
+告诉
+画
+教
+开学
+考
+考试
+旅游
+拿
+跑步
+肉
+试
+送
+踢
+跳舞
+洗
+游
+游泳
+运动
+站
+准备
+花</t>
+  </si>
+  <si>
+    <t>包
+本子
+笔
+床
+蛋糕
+花
+画
+画笔
+机票
+咖啡
+裤子
+篮球
+礼物
+门
+门票
+面
+奶茶
+票
+球
+书包
+足球</t>
+  </si>
+  <si>
+    <t>班
+车站
+饭馆
+房子
+高中
+机场
+教室
+酒店
+楼
+路
+路上
+门口
+商场
+外国
+洗手间
+药店
+站</t>
+  </si>
+  <si>
+    <t>出国
+出门
+出去
+打车
+地铁
+动
+飞
+公交车
+过
+过来
+过去
+回来
+回去
+接
+进
+进来
+进去
+离
+路上
+跑
+跑步
+上来
+上去
+上网
+往
+下来
+下去
+站
+走
+走路
+出</t>
+  </si>
+  <si>
+    <t>出去
+后面
+近
+里面
+门口
+旁边
+前面
+上面
+外面
+网上
+下面
+右
+右边
+远
+左</t>
+  </si>
+  <si>
+    <t>从小
+过年
+经常
+就
+开始
+开学
+快要
+生日
+时
+小时候
+新年
+一会儿
+已经
+有时
+周</t>
+  </si>
+  <si>
+    <t>白色
+不错
+长
+错
+高
+好像
+黑色
+红色
+坏
+近
+快
+慢
+没意思
+晴
+完
+颜色
+阴
+有意思
+远</t>
   </si>
   <si>
     <t>啊
@@ -95,293 +391,6 @@
 最</t>
   </si>
   <si>
-    <t>Ai Là Triệu Phú HSK 2</t>
-  </si>
-  <si>
-    <t>HTML, CSS, Javascript</t>
-  </si>
-  <si>
-    <t>Trắc nghiệm / Trò chơi truyền hình</t>
-  </si>
-  <si>
-    <t>Nhận diện Hán tự, Ghi nhớ nghĩa, Phản xạ từ vựng HSK 2</t>
-  </si>
-  <si>
-    <t>Khởi động 5 phút đầu giờ; Bài tập về nhà; Ôn tập cuối chương</t>
-  </si>
-  <si>
-    <t>Cá nhân, Chia đội thi đấu (Đội nào giành được nhiều tiền hơn), Giáo viên chiếu bảng lớp học</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude1</t>
-  </si>
-  <si>
-    <t>Cảm xúc &amp; Thái độ</t>
-  </si>
-  <si>
-    <t>啊
-爱好
-不错
-不好意思
-坏
-快乐
-没意思
-舒服
-希望
-笑</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude2</t>
-  </si>
-  <si>
-    <t>Đời sống sinh hoạt</t>
-  </si>
-  <si>
-    <t>爱情片
-帮忙
-包
-笔
-打
-打开
-蛋糕
-等
-点
-告诉
-画
-教
-开学
-考
-考试
-旅游
-拿
-跑步
-肉
-试
-送
-踢
-跳舞
-洗
-游
-游泳
-运动
-站
-准备
-花</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude3</t>
-  </si>
-  <si>
-    <t>Miêu tả &amp; Đánh giá</t>
-  </si>
-  <si>
-    <t>白色
-不错
-长
-错
-高
-好像
-黑色
-红色
-坏
-近
-快
-慢
-没意思
-晴
-完
-颜色
-阴
-有意思
-远</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude4</t>
-  </si>
-  <si>
-    <t>Cơ thể &amp; Sức khỏe</t>
-  </si>
-  <si>
-    <t>白色
-帮
-长
-高
-个子
-介绍
-累
-身体
-手
-手表
-疼
-头
-眼睛
-药
-药店</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude5</t>
-  </si>
-  <si>
-    <t>Địa điểm &amp; Nơi chốn</t>
-  </si>
-  <si>
-    <t>班
-车站
-饭馆
-房子
-高中
-机场
-教室
-酒店
-楼
-路
-路上
-门口
-商场
-外国
-洗手间
-药店
-站</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude6</t>
-  </si>
-  <si>
-    <t>Đồ vật &amp; Công cụ</t>
-  </si>
-  <si>
-    <t>包
-本子
-笔
-床
-蛋糕
-花
-画
-画笔
-机票
-咖啡
-裤子
-篮球
-礼物
-门
-门票
-面
-奶茶
-票
-球
-书包
-足球</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude7</t>
-  </si>
-  <si>
-    <t>Giao thông &amp; Di chuyển</t>
-  </si>
-  <si>
-    <t>出国
-出门
-出去
-打车
-地铁
-动
-飞
-公交车
-过
-过来
-过去
-回来
-回去
-接
-进
-进来
-进去
-离
-路上
-跑
-跑步
-上来
-上去
-上网
-往
-下来
-下去
-站
-走
-走路
-出</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude8</t>
-  </si>
-  <si>
-    <t>Không gian &amp; Vị trí</t>
-  </si>
-  <si>
-    <t>出去
-后面
-近
-里面
-门口
-旁边
-前面
-上面
-外面
-网上
-下面
-右
-右边
-远
-左</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude9</t>
-  </si>
-  <si>
-    <t>Thời gian</t>
-  </si>
-  <si>
-    <t>从小
-过年
-经常
-就
-开始
-开学
-快要
-生日
-时
-小时候
-新年
-一会儿
-已经
-有时
-周</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude10</t>
-  </si>
-  <si>
-    <t>Con người &amp; Các mối quan hệ</t>
-  </si>
-  <si>
-    <t>介绍
-奶奶
-男孩儿
-女孩儿
-妻子
-小孩儿
-姓
-姓名
-爷爷
-丈夫</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude11</t>
-  </si>
-  <si>
-    <t>Tự nhiên</t>
-  </si>
-  <si>
     <t>咖啡
 绿色
 鸟
@@ -391,9 +400,6 @@
 鱼
 红茶
 绿茶</t>
-  </si>
-  <si>
-    <t>game.html?topic=chude12</t>
   </si>
 </sst>
 </file>
@@ -773,19 +779,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="30.796875" customWidth="1"/>
     <col min="2" max="2" width="50.796875" customWidth="1"/>
-    <col min="3" max="3" width="30.796875" customWidth="1"/>
-    <col min="4" max="4" width="20.796875" customWidth="1"/>
-    <col min="5" max="5" width="30.796875" customWidth="1"/>
-    <col min="6" max="8" width="50.796875" customWidth="1"/>
-    <col min="9" max="9" width="30.796875" customWidth="1"/>
+    <col min="3" max="3" width="25.796875" customWidth="1"/>
+    <col min="4" max="5" width="20.796875" customWidth="1"/>
+    <col min="6" max="7" width="30.796875" customWidth="1"/>
+    <col min="8" max="8" width="50.796875" customWidth="1"/>
+    <col min="9" max="10" width="60.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -813,13 +819,16 @@
       <c r="I1" t="s">
         <v>8</v>
       </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
     </row>
-    <row r="2" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="156" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="C2" t="s">
         <v>11</v>
@@ -842,13 +851,16 @@
       <c r="I2" t="s">
         <v>17</v>
       </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
     </row>
-    <row r="3" spans="1:9" ht="156" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="234" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s">
         <v>11</v>
@@ -863,21 +875,24 @@
         <v>14</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
         <v>16</v>
       </c>
       <c r="I3" t="s">
-        <v>20</v>
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" ht="156" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>22</v>
+        <v>43</v>
       </c>
       <c r="C4" t="s">
         <v>11</v>
@@ -892,21 +907,24 @@
         <v>14</v>
       </c>
       <c r="G4" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="H4" t="s">
         <v>16</v>
       </c>
       <c r="I4" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" ht="296.39999999999998" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>24</v>
-      </c>
       <c r="B5" s="1" t="s">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
@@ -921,21 +939,24 @@
         <v>14</v>
       </c>
       <c r="G5" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H5" t="s">
         <v>16</v>
       </c>
       <c r="I5" t="s">
-        <v>26</v>
+        <v>17</v>
+      </c>
+      <c r="J5" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="234" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="327.60000000000002" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
@@ -950,21 +971,24 @@
         <v>14</v>
       </c>
       <c r="G6" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="H6" t="s">
         <v>16</v>
       </c>
       <c r="I6" t="s">
-        <v>29</v>
+        <v>17</v>
+      </c>
+      <c r="J6" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="265.2" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="265.2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="C7" t="s">
         <v>11</v>
@@ -979,21 +1003,24 @@
         <v>14</v>
       </c>
       <c r="G7" t="s">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="H7" t="s">
         <v>16</v>
       </c>
       <c r="I7" t="s">
-        <v>32</v>
+        <v>17</v>
+      </c>
+      <c r="J7" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="327.60000000000002" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C8" t="s">
         <v>11</v>
@@ -1008,21 +1035,24 @@
         <v>14</v>
       </c>
       <c r="G8" t="s">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="H8" t="s">
         <v>16</v>
       </c>
       <c r="I8" t="s">
-        <v>35</v>
+        <v>17</v>
+      </c>
+      <c r="J8" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="234" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
         <v>11</v>
@@ -1037,21 +1067,24 @@
         <v>14</v>
       </c>
       <c r="G9" t="s">
-        <v>15</v>
+        <v>32</v>
       </c>
       <c r="H9" t="s">
         <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>38</v>
+        <v>17</v>
+      </c>
+      <c r="J9" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="234" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="234" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>49</v>
       </c>
       <c r="C10" t="s">
         <v>11</v>
@@ -1066,21 +1099,24 @@
         <v>14</v>
       </c>
       <c r="G10" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="H10" t="s">
         <v>16</v>
       </c>
       <c r="I10" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="J10" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="234" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="296.39999999999998" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="C11" t="s">
         <v>11</v>
@@ -1095,21 +1131,24 @@
         <v>14</v>
       </c>
       <c r="G11" t="s">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="H11" t="s">
         <v>16</v>
       </c>
       <c r="I11" t="s">
-        <v>44</v>
+        <v>17</v>
+      </c>
+      <c r="J11" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="156" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
         <v>11</v>
@@ -1124,21 +1163,24 @@
         <v>14</v>
       </c>
       <c r="G12" t="s">
-        <v>15</v>
+        <v>38</v>
       </c>
       <c r="H12" t="s">
         <v>16</v>
       </c>
       <c r="I12" t="s">
-        <v>47</v>
+        <v>17</v>
+      </c>
+      <c r="J12" t="s">
+        <v>18</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="140.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="140.4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="C13" t="s">
         <v>11</v>
@@ -1153,19 +1195,23 @@
         <v>14</v>
       </c>
       <c r="G13" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H13" t="s">
         <v>16</v>
       </c>
       <c r="I13" t="s">
-        <v>50</v>
+        <v>17</v>
+      </c>
+      <c r="J13" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I1 A13 A2 C2:I2 A3 C3:I3 A4 C4:I4 A5 C5:I5 A6 C6:I6 A7 C7:I7 A8 C8:I8 A9 C9:I9 A10 C10:I10 A11 C11:I11 A12 C12:I12 C13:I13" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:J1 A13 A2 C2:J2 A3 C3:J3 A4 C4:J4 A5 C5:J5 A6 C6:J6 A7 C7:J7 A8 C8:J8 A9 C9:J9 A10 C10:J10 A11 C11:J11 A12 C12:J12 C13:J13" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>